<commit_message>
Data update 2026-08-31 11:36
</commit_message>
<xml_diff>
--- a/Database/Database.xlsx
+++ b/Database/Database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://etgworld.sharepoint.com/sites/SoftsDatabase/Shared Documents/Database/Hardmine/Fundamental/Cocoa Pod Counts/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F036B47-78AF-4FD7-8EB4-64B742FED634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="8_{7F036B47-78AF-4FD7-8EB4-64B742FED634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9968BAF-2B1F-4D0F-8259-A8C96691E2CE}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{163F1A64-16DF-4783-B120-E833BAC1395A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4185" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4257" uniqueCount="21">
   <si>
     <t>NUMBER</t>
   </si>
@@ -476,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ED50651-EC6B-4F2C-8FAD-680954E456A8}">
-  <dimension ref="A1:F1394"/>
+  <dimension ref="A1:F1418"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="3" max="3" width="10.47265625" customWidth="1"/>
@@ -3865,7 +3865,7 @@
         <v>1950</v>
       </c>
       <c r="C170" s="1">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="D170" s="1" t="s">
         <v>6</v>
@@ -3885,7 +3885,7 @@
         <v>1950</v>
       </c>
       <c r="C171" s="1">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="D171" s="1" t="s">
         <v>9</v>
@@ -3905,7 +3905,7 @@
         <v>1950</v>
       </c>
       <c r="C172" s="1">
-        <v>9.6</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="D172" s="1" t="s">
         <v>10</v>
@@ -3925,7 +3925,7 @@
         <v>1950</v>
       </c>
       <c r="C173" s="1">
-        <v>11.8</v>
+        <v>12.2</v>
       </c>
       <c r="D173" s="1" t="s">
         <v>11</v>
@@ -3945,7 +3945,7 @@
         <v>1950</v>
       </c>
       <c r="C174" s="1">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="D174" s="1" t="s">
         <v>12</v>
@@ -3965,7 +3965,7 @@
         <v>1950</v>
       </c>
       <c r="C175" s="1">
-        <v>2.2000000000000002</v>
+        <v>1.7</v>
       </c>
       <c r="D175" s="1" t="s">
         <v>13</v>
@@ -4085,7 +4085,7 @@
         <v>1950</v>
       </c>
       <c r="C181" s="1">
-        <v>19.100000000000001</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="D181" s="1" t="s">
         <v>19</v>
@@ -4105,7 +4105,7 @@
         <v>1950</v>
       </c>
       <c r="C182" s="1">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
       <c r="D182" s="1" t="s">
         <v>6</v>
@@ -4125,7 +4125,7 @@
         <v>1950</v>
       </c>
       <c r="C183" s="1">
-        <v>0.8</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="D183" s="1" t="s">
         <v>9</v>
@@ -4145,7 +4145,7 @@
         <v>1950</v>
       </c>
       <c r="C184" s="1">
-        <v>11.1</v>
+        <v>13.4</v>
       </c>
       <c r="D184" s="1" t="s">
         <v>10</v>
@@ -4165,7 +4165,7 @@
         <v>1950</v>
       </c>
       <c r="C185" s="1">
-        <v>11.8</v>
+        <v>15.6</v>
       </c>
       <c r="D185" s="1" t="s">
         <v>11</v>
@@ -4185,7 +4185,7 @@
         <v>1950</v>
       </c>
       <c r="C186" s="1">
-        <v>2.7</v>
+        <v>1.7</v>
       </c>
       <c r="D186" s="1" t="s">
         <v>12</v>
@@ -4205,7 +4205,7 @@
         <v>1950</v>
       </c>
       <c r="C187" s="1">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="D187" s="1" t="s">
         <v>13</v>
@@ -4225,7 +4225,7 @@
         <v>1950</v>
       </c>
       <c r="C188" s="1">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="D188" s="1" t="s">
         <v>14</v>
@@ -4325,7 +4325,7 @@
         <v>1950</v>
       </c>
       <c r="C193" s="1">
-        <v>19</v>
+        <v>20.7</v>
       </c>
       <c r="D193" s="1" t="s">
         <v>19</v>
@@ -28243,6 +28243,470 @@
       </c>
       <c r="F1394" s="1" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="1395" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1395" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1395" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1395" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="D1395" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1395" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1395" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1396" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1396" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1396" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1396" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="D1396" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1396" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1396" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1397" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1397" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1397" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1397" s="1">
+        <v>10.4</v>
+      </c>
+      <c r="D1397" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1397" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1397" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1398" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1398" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1398" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1398" s="1">
+        <v>11.7</v>
+      </c>
+      <c r="D1398" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1398" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1398" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1399" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1399" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1399" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1399" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="D1399" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1399" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1399" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1400" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1400" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1400" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1400" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="D1400" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1400" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1400" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1401" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1401" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1401" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1401" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="D1401" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1401" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1401" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1402" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1402" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1402" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1402" s="1"/>
+      <c r="D1402" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1402" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1402" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1403" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1403" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1403" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1403" s="1"/>
+      <c r="D1403" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1403" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1403" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1404" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1404" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1404" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1404" s="1"/>
+      <c r="D1404" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1404" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1404" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1405" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1405" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1405" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1405" s="1"/>
+      <c r="D1405" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1405" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1405" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1406" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1406" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1406" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1406" s="1">
+        <v>15.4</v>
+      </c>
+      <c r="D1406" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1406" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1406" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1407" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1407" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1407" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1407" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="D1407" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1407" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1407" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1408" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1408" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1408" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1408" s="1">
+        <v>2.6</v>
+      </c>
+      <c r="D1408" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1408" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1408" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1409" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1409" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1409" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1409" s="1">
+        <v>9</v>
+      </c>
+      <c r="D1409" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1409" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1409" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1410" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1410" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1410" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1410" s="1">
+        <v>11.6</v>
+      </c>
+      <c r="D1410" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1410" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1410" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1411" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1411" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1411" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1411" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="D1411" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1411" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1411" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1412" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1412" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1412" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1412" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="D1412" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1412" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1412" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1413" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1413" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1413" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1413" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="D1413" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1413" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1413" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1414" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1414" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1414" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1414" s="1"/>
+      <c r="D1414" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1414" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1414" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1415" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1415" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1415" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1415" s="1"/>
+      <c r="D1415" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1415" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1415" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1416" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1416" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1416" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1416" s="1"/>
+      <c r="D1416" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1416" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1416" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1417" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1417" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1417" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1417" s="1"/>
+      <c r="D1417" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1417" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1417" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1418" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1418" s="1">
+        <v>8</v>
+      </c>
+      <c r="B1418" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1418" s="1">
+        <v>15</v>
+      </c>
+      <c r="D1418" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1418" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1418" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -28251,6 +28715,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3bb8a688-9fce-46e7-b438-b3767c5bce2d" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010069BD0CCD6E02B74F9DAE55BEF75C7D8B" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="755c61f92718ec80af2f84face8369ae">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff" xmlns:ns3="3bb8a688-9fce-46e7-b438-b3767c5bce2d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6db04e3886905a89fbc2397dfd3aa562" ns2:_="" ns3:_="">
     <xsd:import namespace="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff"/>
@@ -28439,36 +28923,42 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3bb8a688-9fce-46e7-b438-b3767c5bce2d" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B67746DD-B886-498E-8677-5A5A601F30FB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A128B452-C6BB-4789-B352-0AE3FCE4DF0E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A128B452-C6BB-4789-B352-0AE3FCE4DF0E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4BD7AE23-D2C3-4D38-8730-9D6ABA1E3C0B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3bb8a688-9fce-46e7-b438-b3767c5bce2d"/>
+    <ds:schemaRef ds:uri="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4BD7AE23-D2C3-4D38-8730-9D6ABA1E3C0B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B67746DD-B886-498E-8677-5A5A601F30FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff"/>
+    <ds:schemaRef ds:uri="3bb8a688-9fce-46e7-b438-b3767c5bce2d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Data update 2026-09-21 11:49
</commit_message>
<xml_diff>
--- a/Database/Database.xlsx
+++ b/Database/Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://etgworld.sharepoint.com/sites/SoftsDatabase/Shared Documents/Database/Hardmine/Fundamental/Cocoa Pod Counts/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="8_{7F036B47-78AF-4FD7-8EB4-64B742FED634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9968BAF-2B1F-4D0F-8259-A8C96691E2CE}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="8_{7F036B47-78AF-4FD7-8EB4-64B742FED634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09C50947-A41D-4E2D-95AB-ACBF9ECE0AAB}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{163F1A64-16DF-4783-B120-E833BAC1395A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4257" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4293" uniqueCount="21">
   <si>
     <t>NUMBER</t>
   </si>
@@ -476,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ED50651-EC6B-4F2C-8FAD-680954E456A8}">
-  <dimension ref="A1:F1418"/>
+  <dimension ref="A1:F1430"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="3" max="3" width="10.47265625" customWidth="1"/>
@@ -4345,7 +4345,7 @@
         <v>1950</v>
       </c>
       <c r="C194" s="1">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D194" s="1" t="s">
         <v>6</v>
@@ -4365,7 +4365,7 @@
         <v>1950</v>
       </c>
       <c r="C195" s="1">
-        <v>1.3</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D195" s="1" t="s">
         <v>9</v>
@@ -4385,7 +4385,7 @@
         <v>1950</v>
       </c>
       <c r="C196" s="1">
-        <v>8.6999999999999993</v>
+        <v>8.9</v>
       </c>
       <c r="D196" s="1" t="s">
         <v>10</v>
@@ -4445,7 +4445,7 @@
         <v>1950</v>
       </c>
       <c r="C199" s="1">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="D199" s="1" t="s">
         <v>13</v>
@@ -4565,7 +4565,7 @@
         <v>1950</v>
       </c>
       <c r="C205" s="1">
-        <v>17.600000000000001</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="D205" s="1" t="s">
         <v>19</v>
@@ -28706,6 +28706,238 @@
         <v>7</v>
       </c>
       <c r="F1418" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1419" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1419" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1419" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1419" s="1">
+        <v>1</v>
+      </c>
+      <c r="D1419" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1419" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1419" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1420" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1420" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1420" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1420" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="D1420" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1420" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1420" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1421" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1421" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1421" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1421" s="1">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="D1421" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1421" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1421" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1422" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1422" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1422" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1422" s="1">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="D1422" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1422" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1422" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1423" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1423" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1423" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1423" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="D1423" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1423" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1423" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1424" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1424" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1424" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1424" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="D1424" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1424" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1424" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1425" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1425" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1425" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1425" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="D1425" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1425" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1425" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1426" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1426" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1426" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1426" s="1"/>
+      <c r="D1426" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1426" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1426" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1427" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1427" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1427" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1427" s="1"/>
+      <c r="D1427" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1427" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1427" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1428" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1428" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1428" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1428" s="1"/>
+      <c r="D1428" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1428" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1428" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1429" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1429" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1429" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1429" s="1"/>
+      <c r="D1429" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1429" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1429" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1430" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1430" s="1">
+        <v>9</v>
+      </c>
+      <c r="B1430" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C1430" s="1">
+        <v>13.4</v>
+      </c>
+      <c r="D1430" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1430" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1430" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -28715,26 +28947,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3bb8a688-9fce-46e7-b438-b3767c5bce2d" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010069BD0CCD6E02B74F9DAE55BEF75C7D8B" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="755c61f92718ec80af2f84face8369ae">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff" xmlns:ns3="3bb8a688-9fce-46e7-b438-b3767c5bce2d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6db04e3886905a89fbc2397dfd3aa562" ns2:_="" ns3:_="">
     <xsd:import namespace="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff"/>
@@ -28923,26 +29135,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A128B452-C6BB-4789-B352-0AE3FCE4DF0E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3bb8a688-9fce-46e7-b438-b3767c5bce2d" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4BD7AE23-D2C3-4D38-8730-9D6ABA1E3C0B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3bb8a688-9fce-46e7-b438-b3767c5bce2d"/>
-    <ds:schemaRef ds:uri="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B67746DD-B886-498E-8677-5A5A601F30FB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -28961,6 +29174,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4BD7AE23-D2C3-4D38-8730-9D6ABA1E3C0B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3bb8a688-9fce-46e7-b438-b3767c5bce2d"/>
+    <ds:schemaRef ds:uri="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A128B452-C6BB-4789-B352-0AE3FCE4DF0E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{9324bd15-b7b3-4e59-b23e-9f53050507bb}" enabled="0" method="" siteId="{9324bd15-b7b3-4e59-b23e-9f53050507bb}" removed="1"/>

</xml_diff>